<commit_message>
problems summary in excel
</commit_message>
<xml_diff>
--- a/movies working.xlsx
+++ b/movies working.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tudublin-my.sharepoint.com/personal/a00043106_mytudublin_ie/Documents/Documents/GitHub/Data-CA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="309" documentId="11_F25DC773A252ABDACC10481131DA6A845ADE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E5511D0-7FA7-43D9-9F76-A4EEC6044BF0}"/>
+  <xr:revisionPtr revIDLastSave="321" documentId="11_F25DC773A252ABDACC10481131DA6A845ADE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D38608A-F4F5-491A-849C-513CB0D44F27}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1051" uniqueCount="630">
   <si>
     <t>title</t>
   </si>
@@ -1924,6 +1924,30 @@
   </si>
   <si>
     <t>gross income num</t>
+  </si>
+  <si>
+    <t>edited</t>
+  </si>
+  <si>
+    <t xml:space="preserve">problems noticed </t>
+  </si>
+  <si>
+    <t>gross total missing values</t>
+  </si>
+  <si>
+    <t>gross total M $ symbols</t>
+  </si>
+  <si>
+    <t>gross total numbers are text</t>
+  </si>
+  <si>
+    <t>certificate "Unrated" as lack of info</t>
+  </si>
+  <si>
+    <t>genre multiple genras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">title unusual name last movie </t>
   </si>
 </sst>
 </file>
@@ -1934,7 +1958,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="173" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1951,18 +1975,30 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1979,23 +2015,26 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="4"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="3"/>
   </cellXfs>
-  <cellStyles count="4">
-    <cellStyle name="Bad" xfId="3" builtinId="27"/>
+  <cellStyles count="5">
+    <cellStyle name="Bad" xfId="4" builtinId="27"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Good" xfId="3" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
@@ -2356,6 +2395,9 @@
       <c r="M2" t="s">
         <v>597</v>
       </c>
+      <c r="Q2" s="6" t="s">
+        <v>622</v>
+      </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -2403,10 +2445,10 @@
       <c r="P3" t="s">
         <v>4</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="Q3" s="6" t="s">
         <v>621</v>
       </c>
-      <c r="R3" s="3" t="s">
+      <c r="R3" t="s">
         <v>598</v>
       </c>
     </row>
@@ -2459,7 +2501,7 @@
         <f>251-COUNTIF(E2:E251, "")</f>
         <v>251</v>
       </c>
-      <c r="Q4">
+      <c r="Q4" s="6">
         <f>251-COUNTIF(J2:J251, "")</f>
         <v>247</v>
       </c>
@@ -2517,11 +2559,11 @@
         <f>COUNTBLANK(E2:E251)/100</f>
         <v>0</v>
       </c>
-      <c r="Q5" s="4">
+      <c r="Q5" s="6">
         <f>COUNTBLANK(J2:J251)/100</f>
         <v>0.04</v>
       </c>
-      <c r="R5" s="4">
+      <c r="R5">
         <f>COUNTBLANK(H2:H251)/100</f>
         <v>0.04</v>
       </c>
@@ -2563,6 +2605,7 @@
       <c r="M6" t="s">
         <v>601</v>
       </c>
+      <c r="Q6" s="6"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -2613,7 +2656,7 @@
         <f>MIN(E2:E251)</f>
         <v>45</v>
       </c>
-      <c r="Q7">
+      <c r="Q7" s="6">
         <f>MIN(J2:J20)</f>
         <v>0.01</v>
       </c>
@@ -2671,7 +2714,7 @@
         <f>_xlfn.QUARTILE.EXC(E2:E251, 1)</f>
         <v>108</v>
       </c>
-      <c r="Q8">
+      <c r="Q8" s="6">
         <f>_xlfn.QUARTILE.EXC(J2:J20, 1)</f>
         <v>48.2</v>
       </c>
@@ -2729,7 +2772,7 @@
         <f>AVERAGE(E2:E251)</f>
         <v>131.93199999999999</v>
       </c>
-      <c r="Q9">
+      <c r="Q9" s="6">
         <f>AVERAGE(J2:J20)</f>
         <v>445.35684210526307</v>
       </c>
@@ -2787,7 +2830,7 @@
         <f>MEDIAN(E2:E251)</f>
         <v>127.5</v>
       </c>
-      <c r="Q10">
+      <c r="Q10" s="6">
         <f>MEDIAN(J2:J20)</f>
         <v>322.16000000000003</v>
       </c>
@@ -2845,7 +2888,7 @@
         <f>_xlfn.QUARTILE.EXC(E2:E251, 3)</f>
         <v>148</v>
       </c>
-      <c r="Q11">
+      <c r="Q11" s="6">
         <f>_xlfn.QUARTILE.EXC(J2:J20, 3)</f>
         <v>839.79</v>
       </c>
@@ -2903,7 +2946,7 @@
         <f>MAX(E2:E251)</f>
         <v>374</v>
       </c>
-      <c r="Q12">
+      <c r="Q12" s="6">
         <f>MAX(J2:J20)</f>
         <v>1148.97</v>
       </c>
@@ -2961,7 +3004,7 @@
         <f>_xlfn.STDEV.P(E2:E251)</f>
         <v>36.474420845299242</v>
       </c>
-      <c r="Q13">
+      <c r="Q13" s="6">
         <f>_xlfn.STDEV.P(J2:J20)</f>
         <v>383.69350764781052</v>
       </c>
@@ -3004,8 +3047,6 @@
       </c>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
-      <c r="Q14" s="3"/>
-      <c r="R14" s="3"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
@@ -3618,6 +3659,12 @@
         <f t="shared" si="0"/>
         <v>517.78</v>
       </c>
+      <c r="M29" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="N29" s="3"/>
+      <c r="O29" s="3"/>
+      <c r="P29" s="3"/>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
@@ -3651,6 +3698,12 @@
         <f t="shared" si="0"/>
         <v>775.4</v>
       </c>
+      <c r="M30" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+      <c r="P30" s="3"/>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
@@ -3684,6 +3737,12 @@
         <f t="shared" si="0"/>
         <v>392.98</v>
       </c>
+      <c r="M31" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="N31" s="3"/>
+      <c r="O31" s="3"/>
+      <c r="P31" s="3"/>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
@@ -3717,8 +3776,14 @@
         <f t="shared" si="0"/>
         <v>360.18</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="M32" s="3" t="s">
+        <v>626</v>
+      </c>
+      <c r="N32" s="3"/>
+      <c r="O32" s="3"/>
+      <c r="P32" s="3"/>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>96</v>
       </c>
@@ -3750,8 +3815,14 @@
         <f t="shared" si="0"/>
         <v>120.1</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="M33" s="3" t="s">
+        <v>627</v>
+      </c>
+      <c r="N33" s="3"/>
+      <c r="O33" s="3"/>
+      <c r="P33" s="3"/>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>99</v>
       </c>
@@ -3783,8 +3854,14 @@
         <f t="shared" si="0"/>
         <v>465.52</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="M34" s="3" t="s">
+        <v>628</v>
+      </c>
+      <c r="N34" s="3"/>
+      <c r="O34" s="3"/>
+      <c r="P34" s="3"/>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>102</v>
       </c>
@@ -3816,8 +3893,14 @@
         <f t="shared" si="0"/>
         <v>262.55</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="M35" s="3" t="s">
+        <v>629</v>
+      </c>
+      <c r="N35" s="3"/>
+      <c r="O35" s="3"/>
+      <c r="P35" s="3"/>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>105</v>
       </c>
@@ -3850,7 +3933,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>108</v>
       </c>
@@ -3883,7 +3966,7 @@
         <v>32.270000000000003</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>111</v>
       </c>
@@ -3916,7 +3999,7 @@
         <v>979.16</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>115</v>
       </c>
@@ -3949,7 +4032,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>118</v>
       </c>
@@ -3982,7 +4065,7 @@
         <v>292.10000000000002</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>120</v>
       </c>
@@ -4015,7 +4098,7 @@
         <v>50.43</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>123</v>
       </c>
@@ -4048,7 +4131,7 @@
         <v>109.68</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>126</v>
       </c>
@@ -4081,7 +4164,7 @@
         <v>6.72</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>129</v>
       </c>
@@ -4114,7 +4197,7 @@
         <v>23.88</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>131</v>
       </c>
@@ -4147,7 +4230,7 @@
         <v>20.329999999999998</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>133</v>
       </c>
@@ -4180,7 +4263,7 @@
         <v>690.82</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>136</v>
       </c>
@@ -4213,7 +4296,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>138</v>
       </c>

</xml_diff>